<commit_message>
fix: Al Khater ton 표준 단계 스냅 적용 (TON_ORDER 기준)
</commit_message>
<xml_diff>
--- a/price-tracking/channels/alkhater/alkhater_ac_prices.xlsx
+++ b/price-tracking/channels/alkhater/alkhater_ac_prices.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1.83</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2.25</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1.78</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1.83</v>
+        <v>2</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2.02</v>
+        <v>2</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1.83</v>
+        <v>2</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1760,7 +1760,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>2.27</v>
+        <v>2.5</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-05-11 12:34</t>
+          <t>2026-05-11 12:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Al Khater 데이터 품질 전면 수정 (Type/Ton/Cold/Portable)
</commit_message>
<xml_diff>
--- a/price-tracking/channels/alkhater/alkhater_ac_prices.xlsx
+++ b/price-tracking/channels/alkhater/alkhater_ac_prices.xlsx
@@ -524,7 +524,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -586,7 +586,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -648,7 +648,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -772,7 +772,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -834,7 +834,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -896,7 +896,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -1187,7 +1187,9 @@
           <t>WWA20K22R</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>Rotary</t>
@@ -1200,7 +1202,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1262,7 +1264,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1324,7 +1326,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -1386,7 +1388,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -1448,7 +1450,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -1510,7 +1512,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -1572,7 +1574,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I19" t="n">
@@ -1634,7 +1636,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -1696,7 +1698,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -1758,7 +1760,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -1820,7 +1822,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I23" t="n">
@@ -1882,7 +1884,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I24" t="n">
@@ -1944,7 +1946,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -2006,7 +2008,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I26" t="n">
@@ -2068,7 +2070,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I27" t="n">
@@ -2130,7 +2132,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I28" t="n">
@@ -2192,7 +2194,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I29" t="n">
@@ -2254,7 +2256,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I30" t="n">
@@ -2316,7 +2318,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I31" t="n">
@@ -2378,7 +2380,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I32" t="n">
@@ -2440,7 +2442,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I33" t="n">
@@ -2502,7 +2504,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I34" t="n">
@@ -2564,7 +2566,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I35" t="n">
@@ -2621,12 +2623,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Split</t>
+          <t>Portable</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I36" t="n">
@@ -2674,7 +2676,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2683,12 +2685,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Split</t>
+          <t>Portable</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I37" t="n">
@@ -2750,7 +2752,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I38" t="n">
@@ -2812,7 +2814,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I39" t="n">
@@ -2874,7 +2876,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I40" t="n">
@@ -2936,7 +2938,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I41" t="n">
@@ -2998,7 +3000,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -3060,7 +3062,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -3122,7 +3124,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I44" t="n">
@@ -3184,7 +3186,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -3246,7 +3248,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -3308,7 +3310,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -3370,7 +3372,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I48" t="n">
@@ -3427,12 +3429,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Split</t>
+          <t>Portable</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I49" t="n">
@@ -3494,7 +3496,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I50" t="n">
@@ -3556,7 +3558,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I51" t="n">
@@ -3618,7 +3620,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I52" t="n">
@@ -3680,7 +3682,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I53" t="n">
@@ -3737,12 +3739,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Split</t>
+          <t>Free Standing</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I54" t="n">
@@ -3804,7 +3806,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I55" t="n">
@@ -3866,7 +3868,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I56" t="n">
@@ -3928,7 +3930,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I57" t="n">
@@ -3990,7 +3992,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I58" t="n">
@@ -4052,7 +4054,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I59" t="n">
@@ -4114,7 +4116,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I60" t="n">
@@ -4176,7 +4178,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I61" t="n">
@@ -4238,7 +4240,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I62" t="n">
@@ -4300,7 +4302,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I63" t="n">
@@ -4362,7 +4364,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I64" t="n">
@@ -4424,7 +4426,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I65" t="n">
@@ -4486,7 +4488,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I66" t="n">
@@ -4548,7 +4550,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I67" t="n">
@@ -4610,7 +4612,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I68" t="n">
@@ -4657,7 +4659,9 @@
           <t>HW-18LME13</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F69" t="inlineStr">
         <is>
           <t>Rotary</t>
@@ -4670,7 +4674,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I69" t="n">
@@ -4732,7 +4736,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I70" t="n">
@@ -4794,7 +4798,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I71" t="n">
@@ -4856,7 +4860,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I72" t="n">
@@ -4918,7 +4922,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I73" t="n">
@@ -4976,7 +4980,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I74" t="n">
@@ -5038,7 +5042,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I75" t="n">
@@ -5100,7 +5104,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I76" t="n">
@@ -5162,7 +5166,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I77" t="n">
@@ -5224,7 +5228,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I78" t="n">
@@ -5286,7 +5290,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I79" t="n">
@@ -5348,7 +5352,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I80" t="n">
@@ -5410,7 +5414,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I81" t="n">
@@ -5472,7 +5476,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I82" t="n">
@@ -5534,7 +5538,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I83" t="n">
@@ -5596,7 +5600,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I84" t="n">
@@ -5658,7 +5662,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I85" t="n">
@@ -5720,7 +5724,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I86" t="n">
@@ -5782,7 +5786,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I87" t="n">
@@ -5844,7 +5848,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I88" t="n">
@@ -5906,7 +5910,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I89" t="n">
@@ -5968,7 +5972,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I90" t="n">
@@ -6030,7 +6034,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I91" t="n">
@@ -6092,7 +6096,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I92" t="n">
@@ -6154,7 +6158,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I93" t="n">
@@ -6216,7 +6220,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I94" t="n">
@@ -6263,7 +6267,9 @@
           <t>LA242C0</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
+      <c r="E95" t="n">
+        <v>2</v>
+      </c>
       <c r="F95" t="inlineStr">
         <is>
           <t>Rotary</t>
@@ -6276,7 +6282,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I95" t="n">
@@ -6338,7 +6344,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I96" t="n">
@@ -6400,7 +6406,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I97" t="n">
@@ -6462,7 +6468,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I98" t="n">
@@ -6520,7 +6526,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I99" t="n">
@@ -6582,7 +6588,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I100" t="n">
@@ -6644,7 +6650,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I101" t="n">
@@ -6706,7 +6712,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I102" t="n">
@@ -6768,7 +6774,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I103" t="n">
@@ -6830,7 +6836,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I104" t="n">
@@ -6892,7 +6898,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I105" t="n">
@@ -6954,7 +6960,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I106" t="n">
@@ -7016,7 +7022,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I107" t="n">
@@ -7078,7 +7084,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I108" t="n">
@@ -7140,7 +7146,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I109" t="n">
@@ -7202,7 +7208,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I110" t="n">
@@ -7264,7 +7270,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I111" t="n">
@@ -7326,7 +7332,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I112" t="n">
@@ -7388,7 +7394,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I113" t="n">
@@ -7450,7 +7456,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I114" t="n">
@@ -7512,7 +7518,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I115" t="n">
@@ -7574,7 +7580,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I116" t="n">
@@ -7621,7 +7627,9 @@
           <t>DSA12C</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
+      <c r="E117" t="n">
+        <v>1</v>
+      </c>
       <c r="F117" t="inlineStr">
         <is>
           <t>Rotary</t>
@@ -7634,7 +7642,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I117" t="n">
@@ -7696,7 +7704,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I118" t="n">
@@ -7743,7 +7751,9 @@
           <t>FW12X2P22</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
+      <c r="E119" t="n">
+        <v>1</v>
+      </c>
       <c r="F119" t="inlineStr">
         <is>
           <t>Rotary</t>
@@ -7756,7 +7766,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I119" t="n">
@@ -7818,7 +7828,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I120" t="n">
@@ -7880,7 +7890,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I121" t="n">
@@ -7937,12 +7947,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Split</t>
+          <t>Portable</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I122" t="n">
@@ -8004,7 +8014,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I123" t="n">
@@ -8066,7 +8076,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I124" t="n">
@@ -8128,7 +8138,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I125" t="n">
@@ -8190,7 +8200,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I126" t="n">
@@ -8252,7 +8262,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I127" t="n">
@@ -8314,7 +8324,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I128" t="n">
@@ -8376,7 +8386,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I129" t="n">
@@ -8438,7 +8448,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I130" t="n">
@@ -8500,7 +8510,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I131" t="n">
@@ -8562,7 +8572,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I132" t="n">
@@ -8624,7 +8634,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I133" t="n">
@@ -8686,7 +8696,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I134" t="n">
@@ -8748,7 +8758,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I135" t="n">
@@ -8810,7 +8820,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I136" t="n">
@@ -8872,7 +8882,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I137" t="n">
@@ -8934,7 +8944,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I138" t="n">
@@ -8996,7 +9006,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I139" t="n">
@@ -9058,7 +9068,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I140" t="n">
@@ -9120,7 +9130,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I141" t="n">
@@ -9182,7 +9192,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I142" t="n">
@@ -9239,12 +9249,12 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Split</t>
+          <t>Portable</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I143" t="n">
@@ -9306,7 +9316,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I144" t="n">
@@ -9368,7 +9378,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I145" t="n">
@@ -9430,7 +9440,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I146" t="n">
@@ -9492,7 +9502,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I147" t="n">
@@ -9554,7 +9564,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I148" t="n">
@@ -9616,7 +9626,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I149" t="n">
@@ -9678,7 +9688,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I150" t="n">
@@ -9740,7 +9750,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I151" t="n">
@@ -9802,7 +9812,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I152" t="n">
@@ -9864,7 +9874,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I153" t="n">
@@ -9926,7 +9936,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I154" t="n">
@@ -9988,7 +9998,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I155" t="n">
@@ -10050,7 +10060,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I156" t="n">
@@ -10108,7 +10118,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I157" t="n">
@@ -10166,7 +10176,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I158" t="n">
@@ -10224,7 +10234,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I159" t="n">
@@ -10282,7 +10292,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I160" t="n">
@@ -10340,7 +10350,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I161" t="n">
@@ -10402,7 +10412,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I162" t="n">
@@ -10464,7 +10474,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I163" t="n">
@@ -10526,7 +10536,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I164" t="n">
@@ -10588,7 +10598,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I165" t="n">
@@ -10645,12 +10655,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Split</t>
+          <t>Free Standing</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Heat &amp; Cool</t>
         </is>
       </c>
       <c r="I166" t="n">
@@ -10707,12 +10717,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>Split</t>
+          <t>Free Standing</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I167" t="n">
@@ -10774,7 +10784,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I168" t="n">
@@ -10836,7 +10846,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I169" t="n">
@@ -10898,7 +10908,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I170" t="n">
@@ -10960,7 +10970,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I171" t="n">
@@ -11022,7 +11032,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Cooling Only</t>
         </is>
       </c>
       <c r="I172" t="n">

</xml_diff>